<commit_message>
ExcelToJson 속도 개선, Google sheet 구조 변경
google sheet id 여러개 기입 가능, api key 파일 위치 변경
</commit_message>
<xml_diff>
--- a/Example/TableManagerUnity/Assets/TableManager/Editor/ExcelFileTemplate.xlsx
+++ b/Example/TableManagerUnity/Assets/TableManager/Editor/ExcelFileTemplate.xlsx
@@ -1,54 +1,93 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitRepo\skyblock\Assets\ATable\Editor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\syncthing-d9\projects\toast-workspace\toast-develop\ToastUnityClient\Assets\TableManager\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D70815-BAC5-4835-A061-20F132AE85BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B24387E-7DC8-417D-BD90-E2986793FAD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5E11AB79-9758-4167-84DC-193AA32355C2}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="#DataTemplate" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>#</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>string</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>note</t>
   </si>
   <si>
     <t>id</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>temp_id</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -56,22 +95,75 @@
       <color theme="0"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="맑은 고딕"/>
-      <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="9"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="9"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="2" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -90,15 +182,49 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -118,7 +244,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -134,7 +260,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -146,7 +272,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -163,7 +289,7 @@
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic Light"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -193,12 +319,29 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -228,6 +371,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -379,29 +539,85 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B883075C-9E33-4EEA-A3B5-981FA643D488}">
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="16384" width="9" style="2"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="1" t="s">
+    <row r="2" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
         <v>2</v>
       </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+    </row>
+    <row r="3" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7"/>
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="1"/>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="3"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Excel 템플릿 파일 수정, update LocalDb
</commit_message>
<xml_diff>
--- a/Example/TableManagerUnity/Assets/TableManager/Editor/ExcelFileTemplate.xlsx
+++ b/Example/TableManagerUnity/Assets/TableManager/Editor/ExcelFileTemplate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\syncthing-d9\projects\toast-workspace\toast-develop\ToastUnityClient\Assets\TableManager\Editor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\github\unity-data-table\Example\TableManagerUnity\Assets\TableManager\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF203428-AFA2-4383-9E68-85F16C6298D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCB4C8D-F14B-4CE7-9607-D0EA0D31AF71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5E11AB79-9758-4167-84DC-193AA32355C2}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,9 +79,16 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="2" tint="-9.9978637043366805E-2"/>
+      <color theme="9" tint="0.39997558519241921"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="9" tint="0.39997558519241921"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="4">
@@ -118,7 +125,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -131,30 +138,23 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color auto="1"/>
@@ -478,7 +478,7 @@
   <dimension ref="A1:P4"/>
   <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15.95" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10" style="6" customWidth="1"/>
+    <col min="1" max="1" width="10" style="4" customWidth="1"/>
     <col min="2" max="16384" width="12.625" style="1"/>
   </cols>
   <sheetData>
@@ -502,23 +502,23 @@
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
     </row>
-    <row r="2" spans="1:16" s="5" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
+    <row r="2" spans="1:16" s="6" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
     </row>
     <row r="3" spans="1:16" s="3" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -548,7 +548,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>OR(A$1="#", $A1="#")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>